<commit_message>
Deliver the bank payment and insurer-direct upload templates
The two new receipt uploads are listed with the other upload routes and their templates are in the delivery folder; the receipts template carries the Commission Amount column. Their screen is Accounts > Receipts > Bulk Upload.
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Receipts_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Receipts_Upload_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
   <si>
     <t xml:space="preserve">Policy Number</t>
   </si>
@@ -21,6 +21,9 @@
     <t xml:space="preserve">Amount</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission Amount</t>
+  </si>
+  <si>
     <t xml:space="preserve">Receipt Date</t>
   </si>
   <si>
@@ -93,6 +96,12 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission part of the Amount on a combined premium-and-commission file; empty or 0 when the row is premium only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commissionAmount, commission</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date YYYY-MM-DD; today when empty (must be in an open period)</t>
   </si>
   <si>
@@ -153,12 +162,6 @@
     <t xml:space="preserve">Accounts &gt; Receipts &gt; Bulk upload</t>
   </si>
   <si>
-    <t xml:space="preserve">API route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POST /api/receipts/bulk-upload (multipart field "file")</t>
-  </si>
-  <si>
     <t xml:space="preserve">File types</t>
   </si>
   <si>
@@ -168,7 +171,7 @@
     <t xml:space="preserve">Row limit</t>
   </si>
   <si>
-    <t xml:space="preserve">Up to 1,000 data rows per file (Configuration setting limits.bulk_upload_max_rows) and 10 MB.</t>
+    <t xml:space="preserve">Up to 1,000 data rows per file and 10 MB.</t>
   </si>
   <si>
     <t xml:space="preserve">Required columns</t>
@@ -207,10 +210,10 @@
     <t xml:space="preserve">Each row issues an official receipt, applies it to the oldest open bills of the policy and posts the collection journal. The receipt date must fall in an open accounting period.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generated by backend/scripts/build-upload-templates.js from the column list the importer itself uses. Do not rename the headers.</t>
+    <t xml:space="preserve">Headers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The headers are the ones the import reads. Do not rename them.</t>
   </si>
 </sst>
 </file>
@@ -218,9 +221,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -247,8 +250,42 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0B2A4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5F6B76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -276,6 +313,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF4CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -307,9 +362,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -330,6 +385,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -339,20 +401,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20" customHeight="1">
+    <row r="1" spans="1:9" ht="20" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -377,15 +440,15 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="0" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="0" t="s">
@@ -394,8 +457,11 @@
       <c r="E2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>13</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -405,7 +471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -418,22 +484,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2">
@@ -441,16 +507,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -458,16 +524,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -475,16 +541,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -492,12 +555,9 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="4" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="0" t="s">
@@ -512,16 +572,19 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="D6" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="E6" s="0" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -529,13 +592,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -543,13 +609,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
@@ -557,16 +623,30 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="0" t="s">
         <v>38</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -576,7 +656,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -585,106 +665,98 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>